<commit_message>
fix version first dental
</commit_message>
<xml_diff>
--- a/MERG HJR/HAJAR ALMAS 1 .xlsx
+++ b/MERG HJR/HAJAR ALMAS 1 .xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc\Desktop\بطاقات\HJR CARD\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Omar\waad_temp_website\MERG HJR\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16DC906E-D8E1-4CDA-83D5-6E07DD61BFCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12210"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="بنغازي" sheetId="1" r:id="rId1"/>
@@ -22,15 +23,6 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
@@ -782,7 +774,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
@@ -790,7 +782,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -798,7 +790,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -806,7 +798,7 @@
       <b/>
       <sz val="18"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -830,7 +822,7 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -1135,46 +1127,6 @@
   </cellStyles>
   <dxfs count="12">
     <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="16"/>
-        <color theme="1"/>
-        <name val="Sakkal Majalla"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
@@ -1281,6 +1233,46 @@
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <name val="Sakkal Majalla"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -1455,22 +1447,22 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A5:K64" totalsRowShown="0" headerRowDxfId="11" tableBorderDxfId="10">
-  <autoFilter ref="A5:K64"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A5:K64" totalsRowShown="0" headerRowDxfId="11" tableBorderDxfId="10">
+  <autoFilter ref="A5:K64" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="11">
-    <tableColumn id="1" name="Column1" dataDxfId="9">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Column1" dataDxfId="9">
       <calculatedColumnFormula>A5+1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" name="Column2" dataDxfId="8"/>
-    <tableColumn id="3" name="Column3" dataDxfId="7"/>
-    <tableColumn id="4" name="Column4" dataDxfId="6"/>
-    <tableColumn id="11" name="Column42" dataDxfId="0"/>
-    <tableColumn id="5" name="Column5" dataDxfId="5"/>
-    <tableColumn id="6" name="Column6" dataDxfId="4"/>
-    <tableColumn id="7" name="Column7" dataDxfId="3"/>
-    <tableColumn id="8" name="Column8" dataDxfId="2"/>
-    <tableColumn id="9" name="Column9" dataDxfId="1"/>
-    <tableColumn id="10" name="Column10"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Column2" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Column3" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Column4" dataDxfId="6"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Column42" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Column5" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Column6" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Column7" dataDxfId="2"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Column8" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Column9" dataDxfId="0"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Column10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1738,27 +1730,27 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <tabColor theme="4" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A2:L70"/>
-  <sheetFormatPr defaultColWidth="15.7109375" defaultRowHeight="20.25" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="15.69921875" defaultRowHeight="20.25" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.85546875" customWidth="1"/>
-    <col min="2" max="2" width="36.7109375" customWidth="1"/>
-    <col min="3" max="3" width="43.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.42578125" customWidth="1"/>
-    <col min="6" max="6" width="17.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.42578125" customWidth="1"/>
-    <col min="9" max="9" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.42578125" customWidth="1"/>
+    <col min="1" max="1" width="8.8984375" customWidth="1"/>
+    <col min="2" max="2" width="36.69921875" customWidth="1"/>
+    <col min="3" max="3" width="43.69921875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.3984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.3984375" customWidth="1"/>
+    <col min="6" max="6" width="17.59765625" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.296875" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.3984375" customWidth="1"/>
+    <col min="9" max="9" width="11.3984375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.3984375" style="4" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.3984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="2"/>
@@ -1805,7 +1797,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="56.25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="54" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>10</v>
       </c>
@@ -1837,7 +1829,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5"/>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -1849,7 +1841,7 @@
       <c r="I7" s="7"/>
       <c r="J7" s="8"/>
     </row>
-    <row r="8" spans="1:11" s="36" customFormat="1" ht="20.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" s="36" customFormat="1" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="29">
         <v>1</v>
       </c>
@@ -1876,7 +1868,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="9" spans="1:11" s="36" customFormat="1" ht="20.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" s="36" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="29">
         <v>2</v>
       </c>
@@ -3227,7 +3219,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:11" s="36" customFormat="1" ht="20.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" s="36" customFormat="1" ht="22.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="29">
         <v>41</v>
       </c>
@@ -3262,7 +3254,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="49" spans="1:11" s="36" customFormat="1" ht="20.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" s="36" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="29">
         <v>42</v>
       </c>
@@ -3295,7 +3287,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="50" spans="1:11" s="36" customFormat="1" ht="20.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" s="36" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="29">
         <v>43</v>
       </c>
@@ -3330,7 +3322,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="51" spans="1:11" s="36" customFormat="1" ht="20.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" s="36" customFormat="1" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="29">
         <v>44</v>
       </c>
@@ -3365,7 +3357,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="52" spans="1:11" s="36" customFormat="1" ht="20.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" s="36" customFormat="1" ht="25.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="29">
         <v>45</v>
       </c>
@@ -3783,7 +3775,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:11" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="38">
         <v>57</v>
       </c>

</xml_diff>